<commit_message>
Update UI + auto stake
</commit_message>
<xml_diff>
--- a/team_mapping.xlsx
+++ b/team_mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maslo\goalmind-pro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF7B438-243A-4B27-AB84-8944F4529417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF68731-2665-4C25-8D96-1152F0D106E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="492">
   <si>
     <t>fd_name</t>
   </si>
@@ -1484,6 +1484,18 @@
   </si>
   <si>
     <t>PEC Zwolle</t>
+  </si>
+  <si>
+    <t>Accrington ST</t>
+  </si>
+  <si>
+    <t>Boston United</t>
+  </si>
+  <si>
+    <t>Exeter City</t>
+  </si>
+  <si>
+    <t>Ayr Utd</t>
   </si>
 </sst>
 </file>
@@ -1898,6 +1910,9 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
+      <c r="B7" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -2127,6 +2142,9 @@
       <c r="A39" t="s">
         <v>39</v>
       </c>
+      <c r="B39" t="s">
+        <v>491</v>
+      </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
@@ -2273,6 +2291,9 @@
       <c r="A58" t="s">
         <v>58</v>
       </c>
+      <c r="B58" t="s">
+        <v>489</v>
+      </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
@@ -2860,6 +2881,9 @@
     <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>133</v>
+      </c>
+      <c r="B133" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>